<commit_message>
Usability help and repair, refurbishment and diagnostics depth
</commit_message>
<xml_diff>
--- a/demo/registers/Distribution_Issues.xlsx
+++ b/demo/registers/Distribution_Issues.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="77">
   <si>
     <t>Code</t>
   </si>
@@ -77,36 +77,39 @@
     <t>I-700</t>
   </si>
   <si>
+    <t>Plant gate</t>
+  </si>
+  <si>
+    <t>Requested</t>
+  </si>
+  <si>
+    <t>I-701</t>
+  </si>
+  <si>
     <t>Substation B</t>
   </si>
   <si>
-    <t>Requested</t>
-  </si>
-  <si>
-    <t>I-701</t>
+    <t>Rejected</t>
+  </si>
+  <si>
+    <t>I-702</t>
+  </si>
+  <si>
+    <t>Ward 4</t>
   </si>
   <si>
     <t>Approved</t>
   </si>
   <si>
-    <t>I-702</t>
+    <t>I-703</t>
+  </si>
+  <si>
+    <t>Farhan</t>
   </si>
   <si>
     <t>Sector 12</t>
   </si>
   <si>
-    <t>Rejected</t>
-  </si>
-  <si>
-    <t>I-703</t>
-  </si>
-  <si>
-    <t>Farhan</t>
-  </si>
-  <si>
-    <t>Plant gate</t>
-  </si>
-  <si>
     <t>Issued</t>
   </si>
   <si>
@@ -119,81 +122,84 @@
     <t>I-706</t>
   </si>
   <si>
+    <t>Anil</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>I-707</t>
+  </si>
+  <si>
+    <t>Gauri</t>
+  </si>
+  <si>
+    <t>I-708</t>
+  </si>
+  <si>
+    <t>I-709</t>
+  </si>
+  <si>
+    <t>I-710</t>
+  </si>
+  <si>
+    <t>I-711</t>
+  </si>
+  <si>
+    <t>I-712</t>
+  </si>
+  <si>
+    <t>I-713</t>
+  </si>
+  <si>
+    <t>I-714</t>
+  </si>
+  <si>
+    <t>I-715</t>
+  </si>
+  <si>
+    <t>Chirag</t>
+  </si>
+  <si>
+    <t>I-716</t>
+  </si>
+  <si>
+    <t>Divya</t>
+  </si>
+  <si>
+    <t>I-717</t>
+  </si>
+  <si>
+    <t>I-718</t>
+  </si>
+  <si>
+    <t>I-719</t>
+  </si>
+  <si>
+    <t>Bhavna</t>
+  </si>
+  <si>
+    <t>I-720</t>
+  </si>
+  <si>
+    <t>I-721</t>
+  </si>
+  <si>
+    <t>I-722</t>
+  </si>
+  <si>
+    <t>I-723</t>
+  </si>
+  <si>
+    <t>Esha</t>
+  </si>
+  <si>
+    <t>I-724</t>
+  </si>
+  <si>
     <t>Harsh</t>
   </si>
   <si>
-    <t>Ward 4</t>
-  </si>
-  <si>
-    <t>I-707</t>
-  </si>
-  <si>
-    <t>I-708</t>
-  </si>
-  <si>
-    <t>I-709</t>
-  </si>
-  <si>
-    <t>I-710</t>
-  </si>
-  <si>
-    <t>I-711</t>
-  </si>
-  <si>
-    <t>Anil</t>
-  </si>
-  <si>
-    <t>I-712</t>
-  </si>
-  <si>
-    <t>I-713</t>
-  </si>
-  <si>
-    <t>I-714</t>
-  </si>
-  <si>
-    <t>I-715</t>
-  </si>
-  <si>
-    <t>I-716</t>
-  </si>
-  <si>
-    <t>I-717</t>
-  </si>
-  <si>
-    <t>I-718</t>
-  </si>
-  <si>
-    <t>I-719</t>
-  </si>
-  <si>
-    <t>Completed</t>
-  </si>
-  <si>
-    <t>I-720</t>
-  </si>
-  <si>
-    <t>Esha</t>
-  </si>
-  <si>
-    <t>I-721</t>
-  </si>
-  <si>
-    <t>I-722</t>
-  </si>
-  <si>
-    <t>Chirag</t>
-  </si>
-  <si>
-    <t>I-723</t>
-  </si>
-  <si>
-    <t>Gauri</t>
-  </si>
-  <si>
-    <t>I-724</t>
-  </si>
-  <si>
     <t>I-725</t>
   </si>
   <si>
@@ -210,9 +216,6 @@
   </si>
   <si>
     <t>I-730</t>
-  </si>
-  <si>
-    <t>Bhavna</t>
   </si>
   <si>
     <t>I-731</t>
@@ -656,7 +659,7 @@
         <v>5</v>
       </c>
       <c r="C2">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="D2" s="1">
         <v>1850</v>
@@ -670,7 +673,7 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D3" s="1">
         <v>640</v>
@@ -684,7 +687,7 @@
         <v>9</v>
       </c>
       <c r="C4">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="D4" s="1">
         <v>410</v>
@@ -698,7 +701,7 @@
         <v>11</v>
       </c>
       <c r="C5">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1">
         <v>25</v>
@@ -712,7 +715,7 @@
         <v>13</v>
       </c>
       <c r="C6">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D6" s="1">
         <v>120</v>
@@ -765,7 +768,7 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -785,206 +788,218 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>37</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
-      </c>
-      <c r="E9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
+      <c r="G9">
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B12" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C12">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F12" t="s">
-        <v>22</v>
+        <v>37</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
         <v>11</v>
       </c>
       <c r="C13">
-        <v>2</v>
-      </c>
-      <c r="D13" t="s">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F14" t="s">
         <v>22</v>
@@ -992,33 +1007,33 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B15" t="s">
         <v>5</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F15" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
         <v>7</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F16" t="s">
         <v>22</v>
@@ -1026,90 +1041,99 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>48</v>
       </c>
       <c r="E17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F17" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B18" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C18">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>50</v>
       </c>
       <c r="E18" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F18" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19" t="s">
         <v>48</v>
       </c>
-      <c r="B19" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19">
-        <v>2</v>
-      </c>
       <c r="E19" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F19" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C20">
         <v>3</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F20" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
       </c>
       <c r="C21">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="E21" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F21" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G21">
         <v>1</v>
@@ -1117,313 +1141,289 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C22">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F22" t="s">
-        <v>31</v>
+        <v>37</v>
+      </c>
+      <c r="G22">
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B23" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C23">
-        <v>4</v>
-      </c>
-      <c r="D23" t="s">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E23" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F23" t="s">
-        <v>51</v>
-      </c>
-      <c r="G23">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C24">
-        <v>5</v>
-      </c>
-      <c r="D24" t="s">
-        <v>56</v>
+        <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C25">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D25" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E25" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F25" t="s">
-        <v>51</v>
-      </c>
-      <c r="G25">
-        <v>3</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B26" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="D26" t="s">
+        <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F26" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C27">
-        <v>2</v>
-      </c>
-      <c r="D27" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>51</v>
-      </c>
-      <c r="G27">
-        <v>2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F28" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B29" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C29">
         <v>5</v>
       </c>
       <c r="E29" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F29" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E30" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F30" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B31" t="s">
         <v>7</v>
       </c>
       <c r="C31">
-        <v>1</v>
-      </c>
-      <c r="D31" t="s">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F31" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B32" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E32" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F32" t="s">
-        <v>51</v>
-      </c>
-      <c r="G32">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C33">
-        <v>5</v>
-      </c>
-      <c r="D33" t="s">
-        <v>53</v>
+        <v>2</v>
       </c>
       <c r="E33" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F33" t="s">
-        <v>51</v>
-      </c>
-      <c r="G33">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B34" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D34" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E34" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F34" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G34">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B35" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C35">
-        <v>2</v>
-      </c>
-      <c r="D35" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="E35" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="F35" t="s">
-        <v>51</v>
-      </c>
-      <c r="G35">
-        <v>1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C36">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="D36" t="s">
+        <v>61</v>
       </c>
       <c r="E36" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="F36" t="s">
-        <v>22</v>
+        <v>37</v>
+      </c>
+      <c r="G36">
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B37" t="s">
         <v>13</v>
@@ -1431,97 +1431,85 @@
       <c r="C37">
         <v>2</v>
       </c>
-      <c r="D37" t="s">
-        <v>53</v>
-      </c>
       <c r="E37" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F37" t="s">
-        <v>51</v>
-      </c>
-      <c r="G37">
-        <v>1</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B38" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C38">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E38" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F38" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
         <v>5</v>
       </c>
       <c r="C39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D39" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E39" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F39" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G39">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B40" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C40">
         <v>2</v>
       </c>
-      <c r="D40" t="s">
-        <v>58</v>
-      </c>
       <c r="E40" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F40" t="s">
-        <v>51</v>
-      </c>
-      <c r="G40">
-        <v>2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E41" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F41" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>